<commit_message>
Linkprüfung Excel via GitHub-Runner
</commit_message>
<xml_diff>
--- a/Q-Rahmen_Uebersicht_Muenchenstein_Wil_Seelisberg_geprueft.xlsx
+++ b/Q-Rahmen_Uebersicht_Muenchenstein_Wil_Seelisberg_geprueft.xlsx
@@ -3067,7 +3067,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -3076,12 +3076,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Natur- und Heimatschutzrecht Uri (kantonale Erlasse)</t>
+          <t>Verordnung betreffend den Schutz von Naturkörpern und Altertümern</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>RB-Nr. verifizieren</t>
+          <t>sGS 271.51</t>
         </is>
       </c>
       <c r="F27" s="94" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Link zeigte auf die Startseite ur.ch; Gesetz über den Natur- und Heimatschutz = RB 10.5101 (Titel lt. Sammlung: «Gesetz über den Natur- und Heimatschutz»)</t>
+          <t>sGS 271.51 ist seit 31.07.2019 aufgehoben; ersetzt durch den Nachfolgeerlass sGS 271.53 (Titel lt. Sammlung: «Verordnung über die Sicherung und Überlieferung von Naturkörpern»)</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -3099,12 +3099,12 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://www.ur.ch</t>
+          <t>https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/271.51</t>
         </is>
       </c>
       <c r="J27" s="95" t="inlineStr">
         <is>
-          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/10.5101</t>
+          <t>https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/271.53</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3115,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Wasserbau-/Naturgefahrenrecht Uri</t>
+          <t>Natur- und Heimatschutzrecht Uri (kantonale Erlasse)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Link zeigte auf die Startseite ur.ch; Wasserbaugesetz Uri (WBG) = RB 40.1211 (Titel lt. Sammlung: «Wasserbaugesetz (WBG)»)</t>
+          <t>Link zeigte auf die Startseite ur.ch; Gesetz über den Natur- und Heimatschutz = RB 10.5101 (Titel lt. Sammlung: «Gesetz über den Natur- und Heimatschutz»)</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="J28" s="95" t="inlineStr">
         <is>
-          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/40.1211</t>
+          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/10.5101</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3163,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3172,12 +3172,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Beitritt Kanton Uri zur IVöB 2019 (Landratsbeschluss vom 15.06.2022)</t>
+          <t>Wasserbau-/Naturgefahrenrecht Uri</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>IVöB: RB 3.3111</t>
+          <t>RB-Nr. verifizieren</t>
         </is>
       </c>
       <c r="F29" s="94" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Link zeigte auf https://www.ur.ch/_doc/337571 (HTTP 200, «Microsoft PowerPoint - 20230508_Schulung_IVöB_Uri final(2).p»); richtig: RB 3.3111 «Interkantonale Vereinbarung über das öffentliche Beschaffungswesen (IVöB)»</t>
+          <t>Link zeigte auf die Startseite ur.ch; Wasserbaugesetz Uri (WBG) = RB 40.1211 (Titel lt. Sammlung: «Wasserbaugesetz (WBG)»)</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -3195,12 +3195,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://www.ur.ch/_doc/337571</t>
+          <t>https://www.ur.ch</t>
         </is>
       </c>
       <c r="J29" s="95" t="inlineStr">
         <is>
-          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/3.3111</t>
+          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/40.1211</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3220,12 +3220,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Gesetz über die Ausnahmen vom Anwendungsbereich der Interkantonalen Vereinbarung über das öffentliche Beschaffungswesen</t>
+          <t>Beitritt Kanton Uri zur IVöB 2019 (Landratsbeschluss vom 15.06.2022)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>RB-Nr. nicht ermittelt</t>
+          <t>IVöB: RB 3.3111</t>
         </is>
       </c>
       <c r="F30" s="94" t="inlineStr">
@@ -3235,7 +3235,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Link zeigte auf eine Schulungspräsentation; Gesetzestext steht in der Abstimmungsbotschaft vom 12.03.2023 (im Rechtsbuch Uri nicht als eigener Erlass geführt)</t>
+          <t>Link zeigte auf https://www.ur.ch/_doc/337571 (HTTP 200, «Microsoft PowerPoint - 20230508_Schulung_IVöB_Uri final(2).p»); richtig: RB 3.3111 «Interkantonale Vereinbarung über das öffentliche Beschaffungswesen (IVöB)»</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="J30" s="95" t="inlineStr">
         <is>
-          <t>https://ur.ch/_doc/320131</t>
+          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/3.3111</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3268,12 +3268,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Reglement über den Vollzug der IVöB (Submissionsreglement)</t>
+          <t>Gesetz über die Ausnahmen vom Anwendungsbereich der Interkantonalen Vereinbarung über das öffentliche Beschaffungswesen</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>RB 3.3115</t>
+          <t>RB-Nr. nicht ermittelt</t>
         </is>
       </c>
       <c r="F31" s="94" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Link zeigte auf https://www.ur.ch/_doc/337571 (HTTP 200, «Microsoft PowerPoint - 20230508_Schulung_IVöB_Uri final(2).p»); richtig: RB 3.3115 «Reglement über den Vollzug der Interkantonalen Vereinbarung über das öffentliche Beschaffungswesen (Submissionsreglement)»</t>
+          <t>Link zeigte auf eine Schulungspräsentation; Gesetzestext steht in der Abstimmungsbotschaft vom 12.03.2023 (im Rechtsbuch Uri nicht als eigener Erlass geführt)</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="J31" s="95" t="inlineStr">
         <is>
-          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/3.3115</t>
+          <t>https://ur.ch/_doc/320131</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3316,12 +3316,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Abwasserreglement</t>
+          <t>Reglement über den Vollzug der IVöB (Submissionsreglement)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>RB 3.3115</t>
         </is>
       </c>
       <c r="F32" s="94" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Link zeigte auf einen Entwurf («vom ____»); geltende Fassung = SRS 7.4.3-6 (Titel lt. Sammlung: «Abwasserreglement»)</t>
+          <t>Link zeigte auf https://www.ur.ch/_doc/337571 (HTTP 200, «Microsoft PowerPoint - 20230508_Schulung_IVöB_Uri final(2).p»); richtig: RB 3.3115 «Reglement über den Vollzug der Interkantonalen Vereinbarung über das öffentliche Beschaffungswesen (Submissionsreglement)»</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -3339,23 +3339,23 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>https://www.stadtwil.ch/storage/8ae27a52e6272acbe7a00ddad257f439fbae9a367f80166a75d97ea28f6771cf</t>
+          <t>https://www.ur.ch/_doc/337571</t>
         </is>
       </c>
       <c r="J32" s="95" t="inlineStr">
         <is>
-          <t>https://wil-sg.tlex.ch/app/de/texts_of_law/7.4.3-6</t>
+          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/3.3115</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2_Q2_Landschaft</t>
+          <t>1_Q1_Rechtsordnung</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>7</v>
+        <v>88</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3364,12 +3364,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>BLN – Bundesinventar der Landschaften und Naturdenkmäler</t>
+          <t>Abwasserreglement</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>VBLN</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F33" s="94" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
+          <t>Link zeigte auf einen Entwurf («vom ____»); geltende Fassung = SRS 7.4.3-6 (Titel lt. Sammlung: «Abwasserreglement»)</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -3387,12 +3387,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
+          <t>https://www.stadtwil.ch/storage/8ae27a52e6272acbe7a00ddad257f439fbae9a367f80166a75d97ea28f6771cf</t>
         </is>
       </c>
       <c r="J33" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
+          <t>https://wil-sg.tlex.ch/app/de/texts_of_law/7.4.3-6</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3403,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3412,12 +3412,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Bundesinventare Moore, Moorlandschaften, Auen, Amphibienlaichgebiete, Trockenwiesen/-weiden (TWW)</t>
+          <t>BLN – Bundesinventar der Landschaften und Naturdenkmäler</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>NHG / Inventarverordnungen</t>
+          <t>VBLN</t>
         </is>
       </c>
       <c r="F34" s="94" t="inlineStr">
@@ -3435,12 +3435,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
         </is>
       </c>
       <c r="J34" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3460,12 +3460,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Jagdbanngebiete, Wasser- und Zugvogelreservate, Smaragd-Gebiete</t>
+          <t>Bundesinventare Moore, Moorlandschaften, Auen, Amphibienlaichgebiete, Trockenwiesen/-weiden (TWW)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>JSG</t>
+          <t>NHG / Inventarverordnungen</t>
         </is>
       </c>
       <c r="F35" s="94" t="inlineStr">
@@ -3483,12 +3483,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
         </is>
       </c>
       <c r="J35" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3499,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3508,12 +3508,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Wildtierkorridore / Landschaftsverbindungen (überregional)</t>
+          <t>Jagdbanngebiete, Wasser- und Zugvogelreservate, Smaragd-Gebiete</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>JSG</t>
         </is>
       </c>
       <c r="F36" s="94" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Layer-ID ch.bafu.fauna-wildtierkorridore_national existiert nicht, richtig: ch.bafu.fauna-wildtierkorridor_national; Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
         </is>
       </c>
       <c r="H36" t="n">
@@ -3531,12 +3531,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridore_national</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
         </is>
       </c>
       <c r="J36" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3547,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3556,12 +3556,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Wald: Waldareal, Waldreservate, Schutzwald (Bundesgeodaten)</t>
+          <t>Wildtierkorridore / Landschaftsverbindungen (überregional)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>WaG</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F37" s="94" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
+          <t>Layer-ID ch.bafu.fauna-wildtierkorridore_national existiert nicht, richtig: ch.bafu.fauna-wildtierkorridor_national; Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
         </is>
       </c>
       <c r="H37" t="n">
@@ -3579,12 +3579,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridore_national</t>
         </is>
       </c>
       <c r="J37" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -3604,12 +3604,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Gewässernetz, Gewässerschutzkarten, Grundwasserschutzzonen (Bundesdienste)</t>
+          <t>Wald: Waldareal, Waldreservate, Schutzwald (Bundesgeodaten)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>GSchG</t>
+          <t>WaG</t>
         </is>
       </c>
       <c r="F38" s="94" t="inlineStr">
@@ -3627,23 +3627,23 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
         </is>
       </c>
       <c r="J38" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3_Q3_Klima_Energie</t>
+          <t>2_Q2_Landschaft</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -3652,12 +3652,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Sonnendach.ch / Sonnenfassade.ch (Solarpotenzial Dächer und Fassaden)</t>
+          <t>Gewässernetz, Gewässerschutzkarten, Grundwasserschutzzonen (Bundesdienste)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>GSchG</t>
         </is>
       </c>
       <c r="F39" s="94" t="inlineStr">
@@ -3675,12 +3675,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
+          <t>https://map.geo.admin.ch</t>
         </is>
       </c>
       <c r="J39" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
+          <t>https://map.geo.admin.ch</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Geothermie-/Erdwärmesonden-Eignung, Windatlas, Wärmenetz-/Fernwärme-Potenzial</t>
+          <t>Sonnendach.ch / Sonnenfassade.ch (Solarpotenzial Dächer und Fassaden)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3723,12 +3723,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
         </is>
       </c>
       <c r="J40" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Gebäude- und Wohnungsregister (GWR): Heizungsart, Energieträger, Baujahr</t>
+          <t>Geothermie-/Erdwärmesonden-Eignung, Windatlas, Wärmenetz-/Fernwärme-Potenzial</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3771,23 +3771,23 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
+          <t>https://map.geo.admin.ch</t>
         </is>
       </c>
       <c r="J41" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
+          <t>https://map.geo.admin.ch</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>4_Q4_Resilienz</t>
+          <t>3_Q3_Klima_Energie</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Gefährdungskarte Oberflächenabfluss (Starkregen)</t>
+          <t>Gebäude- und Wohnungsregister (GWR): Heizungsart, Energieträger, Baujahr</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3811,7 +3811,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Layer-ID ch.bafu.gefahren-oberflaechenabfluss existiert nicht, richtig: ch.bafu.gefaehrdungskarte-oberflaechenabfluss; Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
         </is>
       </c>
       <c r="H42" t="n">
@@ -3819,12 +3819,12 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-oberflaechenabfluss</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
         </is>
       </c>
       <c r="J42" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -3844,7 +3844,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Erdbebengefährdung / Mikrozonierung (SED), SIA 261 Bauwerksklassen</t>
+          <t>Gefährdungskarte Oberflächenabfluss (Starkregen)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
+          <t>Layer-ID ch.bafu.gefahren-oberflaechenabfluss existiert nicht, richtig: ch.bafu.gefaehrdungskarte-oberflaechenabfluss; Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -3867,12 +3867,12 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-oberflaechenabfluss</t>
         </is>
       </c>
       <c r="J43" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
         </is>
       </c>
     </row>
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -3892,12 +3892,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Lärmbelastung (sonBASE), Störfall-Risikokataster, Kataster belasteter Standorte (Bundesbezug)</t>
+          <t>Erdbebengefährdung / Mikrozonierung (SED), SIA 261 Bauwerksklassen</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>USG / StFV / AltlV</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F44" s="94" t="inlineStr">
@@ -3915,12 +3915,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
         </is>
       </c>
       <c r="J44" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -3940,12 +3940,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Kantonale Naturgefahrenkarten SG</t>
+          <t>Lärmbelastung (sonBASE), Störfall-Risikokataster, Kataster belasteter Standorte (Bundesbezug)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>USG / StFV / AltlV</t>
         </is>
       </c>
       <c r="F45" s="94" t="inlineStr">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Kartenzentrum lag rund 6 km südlich von Wil; auf Wil zentriert</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -3963,12 +3963,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>https://www.geoportal.ch/ktsg/map/3502?y=2717572.22&amp;x=1252351.20&amp;scale=50000&amp;rotation=0</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
         </is>
       </c>
       <c r="J45" s="95" t="inlineStr">
         <is>
-          <t>https://www.geoportal.ch/ktsg/map/3502?y=2721138&amp;x=1258009&amp;scale=50000&amp;rotation=0</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Abwasserreglement</t>
+          <t>Kantonale Naturgefahrenkarten SG</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Link zeigte auf einen Entwurf («vom ____»); geltende Fassung = SRS 7.4.3-6 (Titel lt. Sammlung: «Abwasserreglement»)</t>
+          <t>Kartenzentrum lag rund 6 km südlich von Wil; auf Wil zentriert</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -4011,23 +4011,23 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>https://www.stadtwil.ch/storage/8ae27a52e6272acbe7a00ddad257f439fbae9a367f80166a75d97ea28f6771cf</t>
+          <t>https://www.geoportal.ch/ktsg/map/3502?y=2717572.22&amp;x=1252351.20&amp;scale=50000&amp;rotation=0</t>
         </is>
       </c>
       <c r="J46" s="95" t="inlineStr">
         <is>
-          <t>https://wil-sg.tlex.ch/app/de/texts_of_law/7.4.3-6</t>
+          <t>https://www.geoportal.ch/ktsg/map/3502?y=2721138&amp;x=1258009&amp;scale=50000&amp;rotation=0</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>5_Q5_Ortsbild</t>
+          <t>4_Q4_Resilienz</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -4036,12 +4036,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ISOS – Bundesinventar schützenswerter Ortsbilder der Schweiz</t>
+          <t>Abwasserreglement</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>VISOS</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F47" s="94" t="inlineStr">
@@ -4051,7 +4051,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
+          <t>Link zeigte auf einen Entwurf («vom ____»); geltende Fassung = SRS 7.4.3-6 (Titel lt. Sammlung: «Abwasserreglement»)</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -4059,12 +4059,12 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
+          <t>https://www.stadtwil.ch/storage/8ae27a52e6272acbe7a00ddad257f439fbae9a367f80166a75d97ea28f6771cf</t>
         </is>
       </c>
       <c r="J47" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
+          <t>https://wil-sg.tlex.ch/app/de/texts_of_law/7.4.3-6</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -4084,12 +4084,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>IVS – Inventar historischer Verkehrswege der Schweiz</t>
+          <t>ISOS – Bundesinventar schützenswerter Ortsbilder der Schweiz</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>VIVS</t>
+          <t>VISOS</t>
         </is>
       </c>
       <c r="F48" s="94" t="inlineStr">
@@ -4107,12 +4107,12 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
         </is>
       </c>
       <c r="J48" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -4132,12 +4132,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>KGS-Inventar (Kulturgüter von nationaler/regionaler Bedeutung)</t>
+          <t>IVS – Inventar historischer Verkehrswege der Schweiz</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>VIVS</t>
         </is>
       </c>
       <c r="F49" s="94" t="inlineStr">
@@ -4155,12 +4155,12 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
         </is>
       </c>
       <c r="J49" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -4180,12 +4180,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>BLN (Landschaftsbild / Kulturlandschaft) – Querbezug Q2</t>
+          <t>KGS-Inventar (Kulturgüter von nationaler/regionaler Bedeutung)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>VBLN</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F50" s="94" t="inlineStr">
@@ -4203,23 +4203,23 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
         </is>
       </c>
       <c r="J50" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>6_Q6_Bestellung</t>
+          <t>5_Q5_Ortsbild</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -4228,12 +4228,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>IVöB 2019 inkl. Schwellenwerte</t>
+          <t>BLN (Landschaftsbild / Kulturlandschaft) – Querbezug Q2</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>VBLN</t>
         </is>
       </c>
       <c r="F51" s="94" t="inlineStr">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>PDF war die alte IVöB vom 15.03.2001; ersetzt durch die IVöB-2019-Seite der BPUK</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ statt auf den angezeigten Link</t>
         </is>
       </c>
       <c r="H51" t="n">
@@ -4251,12 +4251,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>https://www.bpuk.ch/fileadmin/Dokumente/bpuk/public/de/konkordate/ivoeb/INTERKANTONALE%2BVEREINBARUNG%2B%25c3%259cBER%2BDAS%2B%25c3%2596FFENTLICHE%2BBESCHAFFUNGSWESEN%2B%28IV%25c3%25b6B%29.pdf</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
         </is>
       </c>
       <c r="J51" s="95" t="inlineStr">
         <is>
-          <t>https://www.bpuk.ch/bpuk/konkordate/ivoeb/ivoeb-2019</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
         </is>
       </c>
     </row>
@@ -4267,7 +4267,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>EG IVöB BL (Gesetz) und kantonale Beschaffungsleitfäden</t>
+          <t>IVöB 2019 inkl. Schwellenwerte</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -4291,20 +4291,20 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Link zeigte auf die Startseite baselland.ch; EG IVöB BL = SGS 420 (Titel lt. Sammlung: «Einführungsgesetz zur interkantonalen Vereinbarung über das öffentliche Beschaffungswesen (EG IVöB)»)</t>
+          <t>PDF war die alte IVöB vom 15.03.2001; ersetzt durch die IVöB-2019-Seite der BPUK</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>403</v>
+        <v>200</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>https://www.baselland.ch</t>
+          <t>https://www.bpuk.ch/fileadmin/Dokumente/bpuk/public/de/konkordate/ivoeb/INTERKANTONALE%2BVEREINBARUNG%2B%25c3%259cBER%2BDAS%2B%25c3%2596FFENTLICHE%2BBESCHAFFUNGSWESEN%2B%28IV%25c3%25b6B%29.pdf</t>
         </is>
       </c>
       <c r="J52" s="95" t="inlineStr">
         <is>
-          <t>https://bl.clex.ch/app/de/texts_of_law/420</t>
+          <t>https://www.bpuk.ch/bpuk/konkordate/ivoeb/ivoeb-2019</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -4324,12 +4324,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>PBG SG: Sondernutzungsplanung / Qualitätsverfahren</t>
+          <t>EG IVöB BL (Gesetz) und kantonale Beschaffungsleitfäden</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>sGS 731.1</t>
+          <t>–</t>
         </is>
       </c>
       <c r="F53" s="94" t="inlineStr">
@@ -4339,20 +4339,20 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Link auf Standardform der Sammlung vereinheitlicht (731.1 «Planungs- und Baugesetz (PBG)»)</t>
+          <t>Link zeigte auf die Startseite baselland.ch; EG IVöB BL = SGS 420 (Titel lt. Sammlung: «Einführungsgesetz zur interkantonalen Vereinbarung über das öffentliche Beschaffungswesen (EG IVöB)»)</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>200</v>
+        <v>403</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>https://www.gesetzessammlung.sg.ch/data/731.1/de</t>
+          <t>https://www.baselland.ch</t>
         </is>
       </c>
       <c r="J53" s="95" t="inlineStr">
         <is>
-          <t>https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/731.1</t>
+          <t>https://bl.clex.ch/app/de/texts_of_law/420</t>
         </is>
       </c>
     </row>
@@ -4363,7 +4363,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -4372,12 +4372,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Beitritt Kanton Uri zur IVöB 2019 (Landratsbeschluss vom 15.06.2022)</t>
+          <t>PBG SG: Sondernutzungsplanung / Qualitätsverfahren</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>IVöB: RB 3.3111</t>
+          <t>sGS 731.1</t>
         </is>
       </c>
       <c r="F54" s="94" t="inlineStr">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Link zeigte auf https://www.ur.ch/_doc/337571 (HTTP 200, «Microsoft PowerPoint - 20230508_Schulung_IVöB_Uri final(2).p»); richtig: RB 3.3111 «Interkantonale Vereinbarung über das öffentliche Beschaffungswesen (IVöB)»</t>
+          <t>Link auf Standardform der Sammlung vereinheitlicht (731.1 «Planungs- und Baugesetz (PBG)»)</t>
         </is>
       </c>
       <c r="H54" t="n">
@@ -4395,12 +4395,12 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>https://www.ur.ch/_doc/337571</t>
+          <t>https://www.gesetzessammlung.sg.ch/data/731.1/de</t>
         </is>
       </c>
       <c r="J54" s="95" t="inlineStr">
         <is>
-          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/3.3111</t>
+          <t>https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/731.1</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -4420,12 +4420,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Gesetz über die Ausnahmen vom Anwendungsbereich der Interkantonalen Vereinbarung über das öffentliche Beschaffungswesen</t>
+          <t>Beitritt Kanton Uri zur IVöB 2019 (Landratsbeschluss vom 15.06.2022)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>RB-Nr. nicht ermittelt</t>
+          <t>IVöB: RB 3.3111</t>
         </is>
       </c>
       <c r="F55" s="94" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Link zeigte auf eine Schulungspräsentation; Gesetzestext steht in der Abstimmungsbotschaft vom 12.03.2023 (im Rechtsbuch Uri nicht als eigener Erlass geführt)</t>
+          <t>Link zeigte auf https://www.ur.ch/_doc/337571 (HTTP 200, «Microsoft PowerPoint - 20230508_Schulung_IVöB_Uri final(2).p»); richtig: RB 3.3111 «Interkantonale Vereinbarung über das öffentliche Beschaffungswesen (IVöB)»</t>
         </is>
       </c>
       <c r="H55" t="n">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="J55" s="95" t="inlineStr">
         <is>
-          <t>https://ur.ch/_doc/320131</t>
+          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/3.3111</t>
         </is>
       </c>
     </row>
@@ -4459,7 +4459,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -4468,12 +4468,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Reglement über den Vollzug der IVöB (Submissionsreglement)</t>
+          <t>Gesetz über die Ausnahmen vom Anwendungsbereich der Interkantonalen Vereinbarung über das öffentliche Beschaffungswesen</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>RB 3.3115</t>
+          <t>RB-Nr. nicht ermittelt</t>
         </is>
       </c>
       <c r="F56" s="94" t="inlineStr">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Link zeigte auf https://www.ur.ch/_doc/337571 (HTTP 200, «Microsoft PowerPoint - 20230508_Schulung_IVöB_Uri final(2).p»); richtig: RB 3.3115 «Reglement über den Vollzug der Interkantonalen Vereinbarung über das öffentliche Beschaffungswesen (Submissionsreglement)»</t>
+          <t>Link zeigte auf eine Schulungspräsentation; Gesetzestext steht in der Abstimmungsbotschaft vom 12.03.2023 (im Rechtsbuch Uri nicht als eigener Erlass geführt)</t>
         </is>
       </c>
       <c r="H56" t="n">
@@ -4496,32 +4496,32 @@
       </c>
       <c r="J56" s="95" t="inlineStr">
         <is>
-          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/3.3115</t>
+          <t>https://ur.ch/_doc/320131</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>7_GIS_Layers</t>
+          <t>6_Q6_Bestellung</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>BLN – Landschaften und Naturdenkmäler von nationaler Bedeutung</t>
+          <t>Reglement über den Vollzug der IVöB (Submissionsreglement)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ch.bafu.bundesinventare-bln</t>
+          <t>RB 3.3115</t>
         </is>
       </c>
       <c r="F57" s="94" t="inlineStr">
@@ -4531,7 +4531,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
+          <t>Link zeigte auf https://www.ur.ch/_doc/337571 (HTTP 200, «Microsoft PowerPoint - 20230508_Schulung_IVöB_Uri final(2).p»); richtig: RB 3.3115 «Reglement über den Vollzug der Interkantonalen Vereinbarung über das öffentliche Beschaffungswesen (Submissionsreglement)»</t>
         </is>
       </c>
       <c r="H57" t="n">
@@ -4539,12 +4539,12 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/</t>
+          <t>https://www.ur.ch/_doc/337571</t>
         </is>
       </c>
       <c r="J57" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
+          <t>https://rechtsbuch.ur.ch/app/de/texts_of_law/3.3115</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -4592,7 +4592,7 @@
       </c>
       <c r="J58" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
         </is>
       </c>
     </row>
@@ -4607,7 +4607,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4640,7 +4640,7 @@
       </c>
       <c r="J59" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4655,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="J60" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
         </is>
       </c>
     </row>
@@ -4699,21 +4699,21 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Moorlandschaften von besonderer Schönheit</t>
+          <t>BLN – Landschaften und Naturdenkmäler von nationaler Bedeutung</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ch.bafu.bundesinventare-moorlandschaften</t>
+          <t>ch.bafu.bundesinventare-bln</t>
         </is>
       </c>
       <c r="F61" s="94" t="inlineStr">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="J61" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-moorlandschaften</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-bln</t>
         </is>
       </c>
     </row>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="J62" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-moorlandschaften</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-moorlandschaften</t>
         </is>
       </c>
     </row>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="J63" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-moorlandschaften</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-moorlandschaften</t>
         </is>
       </c>
     </row>
@@ -4847,7 +4847,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="J64" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-moorlandschaften</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-moorlandschaften</t>
         </is>
       </c>
     </row>
@@ -4891,21 +4891,21 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Hochmoore</t>
+          <t>Moorlandschaften von besonderer Schönheit</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ch.bafu.bundesinventare-hochmoore</t>
+          <t>ch.bafu.bundesinventare-moorlandschaften</t>
         </is>
       </c>
       <c r="F65" s="94" t="inlineStr">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="J65" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-moorlandschaften</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="J66" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="J67" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="J68" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
         </is>
       </c>
     </row>
@@ -5083,21 +5083,21 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Flachmoore</t>
+          <t>Hochmoore</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>ch.bafu.bundesinventare-flachmoore</t>
+          <t>ch.bafu.bundesinventare-hochmoore</t>
         </is>
       </c>
       <c r="F69" s="94" t="inlineStr">
@@ -5120,7 +5120,7 @@
       </c>
       <c r="J69" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-flachmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-hochmoore</t>
         </is>
       </c>
     </row>
@@ -5135,7 +5135,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="J70" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-flachmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-flachmoore</t>
         </is>
       </c>
     </row>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -5216,7 +5216,7 @@
       </c>
       <c r="J71" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-flachmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-flachmoore</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5231,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J72" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-flachmoore</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-flachmoore</t>
         </is>
       </c>
     </row>
@@ -5275,21 +5275,21 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Auengebiete</t>
+          <t>Flachmoore</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ch.bafu.bundesinventare-auen</t>
+          <t>ch.bafu.bundesinventare-flachmoore</t>
         </is>
       </c>
       <c r="F73" s="94" t="inlineStr">
@@ -5312,7 +5312,7 @@
       </c>
       <c r="J73" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-auen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-flachmoore</t>
         </is>
       </c>
     </row>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="J74" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-auen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-auen</t>
         </is>
       </c>
     </row>
@@ -5375,7 +5375,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="J75" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-auen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-auen</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="J76" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-auen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-auen</t>
         </is>
       </c>
     </row>
@@ -5467,21 +5467,21 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Amphibienlaichgebiete (ortsfest)</t>
+          <t>Auengebiete</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>ch.bafu.bundesinventare-amphibien</t>
+          <t>ch.bafu.bundesinventare-auen</t>
         </is>
       </c>
       <c r="F77" s="94" t="inlineStr">
@@ -5504,7 +5504,7 @@
       </c>
       <c r="J77" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-amphibien</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-auen</t>
         </is>
       </c>
     </row>
@@ -5519,7 +5519,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="J78" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-amphibien</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-amphibien</t>
         </is>
       </c>
     </row>
@@ -5567,7 +5567,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="J79" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-amphibien</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-amphibien</t>
         </is>
       </c>
     </row>
@@ -5615,7 +5615,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="J80" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-amphibien</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-amphibien</t>
         </is>
       </c>
     </row>
@@ -5659,21 +5659,21 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Trockenwiesen und -weiden (TWW)</t>
+          <t>Amphibienlaichgebiete (ortsfest)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
+          <t>ch.bafu.bundesinventare-amphibien</t>
         </is>
       </c>
       <c r="F81" s="94" t="inlineStr">
@@ -5696,7 +5696,7 @@
       </c>
       <c r="J81" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-amphibien</t>
         </is>
       </c>
     </row>
@@ -5711,7 +5711,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5744,7 +5744,7 @@
       </c>
       <c r="J82" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
         </is>
       </c>
     </row>
@@ -5759,7 +5759,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="J83" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="J84" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
         </is>
       </c>
     </row>
@@ -5851,21 +5851,21 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Eidg. Jagdbanngebiete</t>
+          <t>Trockenwiesen und -weiden (TWW)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ch.bafu.bundesinventare-jagdbanngebiete</t>
+          <t>ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
         </is>
       </c>
       <c r="F85" s="94" t="inlineStr">
@@ -5888,7 +5888,7 @@
       </c>
       <c r="J85" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-trockenwiesen_trockenweiden</t>
         </is>
       </c>
     </row>
@@ -5903,7 +5903,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5936,7 +5936,7 @@
       </c>
       <c r="J86" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
         </is>
       </c>
     </row>
@@ -5951,7 +5951,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5984,7 +5984,7 @@
       </c>
       <c r="J87" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
         </is>
       </c>
     </row>
@@ -5999,7 +5999,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="J88" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
         </is>
       </c>
     </row>
@@ -6043,21 +6043,21 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Wasser- und Zugvogelreservate</t>
+          <t>Eidg. Jagdbanngebiete</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ch.bafu.bundesinventare-jagdbanngebiete</t>
         </is>
       </c>
       <c r="F89" s="94" t="inlineStr">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Layer-ID ergänzt (ch.bafu.bundesinventare-vogelreservate, «Wasser- und Zugvogelreservate»); Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
         </is>
       </c>
       <c r="H89" t="n">
@@ -6080,7 +6080,7 @@
       </c>
       <c r="J89" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-vogelreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-jagdbanngebiete</t>
         </is>
       </c>
     </row>
@@ -6095,7 +6095,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="J90" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-vogelreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-vogelreservate</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="J91" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-vogelreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-vogelreservate</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6191,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="J92" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-vogelreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-vogelreservate</t>
         </is>
       </c>
     </row>
@@ -6235,21 +6235,21 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Wildtierkorridore (überregional)</t>
+          <t>Wasser- und Zugvogelreservate</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>ch.bafu.fauna-wildtierkorridore_national</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F93" s="94" t="inlineStr">
@@ -6259,7 +6259,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Layer-ID korrigiert (ch.bafu.fauna-wildtierkorridore_national existiert nicht); Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
+          <t>Layer-ID ergänzt (ch.bafu.bundesinventare-vogelreservate, «Wasser- und Zugvogelreservate»); Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
         </is>
       </c>
       <c r="H93" t="n">
@@ -6272,7 +6272,7 @@
       </c>
       <c r="J93" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.bundesinventare-vogelreservate</t>
         </is>
       </c>
     </row>
@@ -6287,7 +6287,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="J94" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6368,7 +6368,7 @@
       </c>
       <c r="J95" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6416,7 +6416,7 @@
       </c>
       <c r="J96" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
         </is>
       </c>
     </row>
@@ -6427,21 +6427,21 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Waldreservate</t>
+          <t>Wildtierkorridore (überregional)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>ch.bafu.waldreservate</t>
+          <t>ch.bafu.fauna-wildtierkorridore_national</t>
         </is>
       </c>
       <c r="F97" s="94" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
+          <t>Layer-ID korrigiert (ch.bafu.fauna-wildtierkorridore_national existiert nicht); Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
         </is>
       </c>
       <c r="H97" t="n">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="J97" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.fauna-wildtierkorridor_national</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6479,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6512,7 +6512,7 @@
       </c>
       <c r="J98" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
         </is>
       </c>
     </row>
@@ -6527,7 +6527,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6560,7 +6560,7 @@
       </c>
       <c r="J99" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
         </is>
       </c>
     </row>
@@ -6575,7 +6575,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="J100" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
         </is>
       </c>
     </row>
@@ -6619,21 +6619,21 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Waldareal / Schutzwald</t>
+          <t>Waldreservate</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ch.bafu.waldreservate</t>
         </is>
       </c>
       <c r="F101" s="94" t="inlineStr">
@@ -6643,7 +6643,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten); keine eindeutige Layer-ID; Link zeigt die Gemeinde ohne Layer</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
         </is>
       </c>
       <c r="H101" t="n">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="J101" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.waldreservate</t>
         </is>
       </c>
     </row>
@@ -6671,7 +6671,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="J102" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6719,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="J103" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -6767,7 +6767,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J104" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -6811,21 +6811,21 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Bauzonen Schweiz (harmonisiert)</t>
+          <t>Waldareal / Schutzwald</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>ch.are.bauzonen</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F105" s="94" t="inlineStr">
@@ -6835,7 +6835,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten); keine eindeutige Layer-ID; Link zeigt die Gemeinde ohne Layer</t>
         </is>
       </c>
       <c r="H105" t="n">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="J105" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.bauzonen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -6863,7 +6863,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6896,7 +6896,7 @@
       </c>
       <c r="J106" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.bauzonen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.bauzonen</t>
         </is>
       </c>
     </row>
@@ -6911,7 +6911,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6944,7 +6944,7 @@
       </c>
       <c r="J107" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.bauzonen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.bauzonen</t>
         </is>
       </c>
     </row>
@@ -6959,7 +6959,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6992,7 +6992,7 @@
       </c>
       <c r="J108" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.bauzonen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.bauzonen</t>
         </is>
       </c>
     </row>
@@ -7003,21 +7003,21 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Solarenergie: Eignung Dächer</t>
+          <t>Bauzonen Schweiz (harmonisiert)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>ch.bfe.solarenergie-eignung-daecher</t>
+          <t>ch.are.bauzonen</t>
         </is>
       </c>
       <c r="F109" s="94" t="inlineStr">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="J109" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.bauzonen</t>
         </is>
       </c>
     </row>
@@ -7055,7 +7055,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="J110" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
         </is>
       </c>
     </row>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7136,7 +7136,7 @@
       </c>
       <c r="J111" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
         </is>
       </c>
     </row>
@@ -7151,7 +7151,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="J112" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
         </is>
       </c>
     </row>
@@ -7195,21 +7195,21 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Solarenergie: Eignung Fassaden</t>
+          <t>Solarenergie: Eignung Dächer</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>ch.bfe.solarenergie-eignung-fassaden</t>
+          <t>ch.bfe.solarenergie-eignung-daecher</t>
         </is>
       </c>
       <c r="F113" s="94" t="inlineStr">
@@ -7232,7 +7232,7 @@
       </c>
       <c r="J113" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-fassaden</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-daecher</t>
         </is>
       </c>
     </row>
@@ -7247,7 +7247,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="J114" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-fassaden</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-fassaden</t>
         </is>
       </c>
     </row>
@@ -7295,7 +7295,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7328,7 +7328,7 @@
       </c>
       <c r="J115" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-fassaden</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-fassaden</t>
         </is>
       </c>
     </row>
@@ -7343,7 +7343,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J116" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-fassaden</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-fassaden</t>
         </is>
       </c>
     </row>
@@ -7387,21 +7387,21 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Gebäude- und Wohnungsregister (Heizung, Energieträger)</t>
+          <t>Solarenergie: Eignung Fassaden</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>ch.bfs.gebaeude_wohnungs_register</t>
+          <t>ch.bfe.solarenergie-eignung-fassaden</t>
         </is>
       </c>
       <c r="F117" s="94" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="J117" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfe.solarenergie-eignung-fassaden</t>
         </is>
       </c>
     </row>
@@ -7439,7 +7439,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7472,7 +7472,7 @@
       </c>
       <c r="J118" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
         </is>
       </c>
     </row>
@@ -7487,7 +7487,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="J119" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
         </is>
       </c>
     </row>
@@ -7535,7 +7535,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7568,7 +7568,7 @@
       </c>
       <c r="J120" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
         </is>
       </c>
     </row>
@@ -7579,21 +7579,21 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Windenergie / Geothermie / Wärmenetz-Potenzial</t>
+          <t>Gebäude- und Wohnungsregister (Heizung, Energieträger)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ch.bfs.gebaeude_wohnungs_register</t>
         </is>
       </c>
       <c r="F121" s="94" t="inlineStr">
@@ -7603,7 +7603,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten); keine eindeutige Layer-ID; Link zeigt die Gemeinde ohne Layer</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
         </is>
       </c>
       <c r="H121" t="n">
@@ -7616,7 +7616,7 @@
       </c>
       <c r="J121" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bfs.gebaeude_wohnungs_register</t>
         </is>
       </c>
     </row>
@@ -7631,7 +7631,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="J122" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -7679,7 +7679,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="J123" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -7727,7 +7727,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="J124" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -7771,21 +7771,21 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>ÖV-Güteklassen</t>
+          <t>Windenergie / Geothermie / Wärmenetz-Potenzial</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>ch.are.gueteklassen_oev</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F125" s="94" t="inlineStr">
@@ -7795,7 +7795,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten); keine eindeutige Layer-ID; Link zeigt die Gemeinde ohne Layer</t>
         </is>
       </c>
       <c r="H125" t="n">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="J125" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.gueteklassen_oev</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -7823,7 +7823,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -7856,7 +7856,7 @@
       </c>
       <c r="J126" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.gueteklassen_oev</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.gueteklassen_oev</t>
         </is>
       </c>
     </row>
@@ -7871,7 +7871,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="J127" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.gueteklassen_oev</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.gueteklassen_oev</t>
         </is>
       </c>
     </row>
@@ -7919,7 +7919,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -7952,7 +7952,7 @@
       </c>
       <c r="J128" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.gueteklassen_oev</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.gueteklassen_oev</t>
         </is>
       </c>
     </row>
@@ -7963,21 +7963,21 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Gefahrenkarten / Gefahrenhinweiskarte (Daten der Kantone)</t>
+          <t>ÖV-Güteklassen</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ch.are.gueteklassen_oev</t>
         </is>
       </c>
       <c r="F129" s="94" t="inlineStr">
@@ -7987,7 +7987,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten); keine eindeutige Layer-ID; Link zeigt die Gemeinde ohne Layer</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
         </is>
       </c>
       <c r="H129" t="n">
@@ -8000,7 +8000,7 @@
       </c>
       <c r="J129" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.are.gueteklassen_oev</t>
         </is>
       </c>
     </row>
@@ -8015,7 +8015,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -8048,7 +8048,7 @@
       </c>
       <c r="J130" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -8063,7 +8063,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -8096,7 +8096,7 @@
       </c>
       <c r="J131" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -8111,7 +8111,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="J132" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -8155,21 +8155,21 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Gefährdungskarte Oberflächenabfluss</t>
+          <t>Gefahrenkarten / Gefahrenhinweiskarte (Daten der Kantone)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>ch.bafu.gefahren-oberflaechenabfluss</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F133" s="94" t="inlineStr">
@@ -8179,7 +8179,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Layer-ID korrigiert (ch.bafu.gefahren-oberflaechenabfluss existiert nicht); Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten); keine eindeutige Layer-ID; Link zeigt die Gemeinde ohne Layer</t>
         </is>
       </c>
       <c r="H133" t="n">
@@ -8192,7 +8192,7 @@
       </c>
       <c r="J133" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -8207,7 +8207,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -8240,7 +8240,7 @@
       </c>
       <c r="J134" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
         </is>
       </c>
     </row>
@@ -8255,7 +8255,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -8288,7 +8288,7 @@
       </c>
       <c r="J135" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
         </is>
       </c>
     </row>
@@ -8303,7 +8303,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="J136" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
         </is>
       </c>
     </row>
@@ -8347,21 +8347,21 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Baugrundklassen (Erdbeben)</t>
+          <t>Gefährdungskarte Oberflächenabfluss</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>ch.bafu.gefahren-baugrundklassen</t>
+          <t>ch.bafu.gefahren-oberflaechenabfluss</t>
         </is>
       </c>
       <c r="F137" s="94" t="inlineStr">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
+          <t>Layer-ID korrigiert (ch.bafu.gefahren-oberflaechenabfluss existiert nicht); Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
         </is>
       </c>
       <c r="H137" t="n">
@@ -8384,7 +8384,7 @@
       </c>
       <c r="J137" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefaehrdungskarte-oberflaechenabfluss</t>
         </is>
       </c>
     </row>
@@ -8399,7 +8399,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -8432,7 +8432,7 @@
       </c>
       <c r="J138" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
         </is>
       </c>
     </row>
@@ -8447,7 +8447,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -8480,7 +8480,7 @@
       </c>
       <c r="J139" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
         </is>
       </c>
     </row>
@@ -8495,7 +8495,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="J140" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
         </is>
       </c>
     </row>
@@ -8539,21 +8539,21 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Strassenlärm Tag</t>
+          <t>Baugrundklassen (Erdbeben)</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>ch.bafu.laerm-strassenlaerm_tag</t>
+          <t>ch.bafu.gefahren-baugrundklassen</t>
         </is>
       </c>
       <c r="F141" s="94" t="inlineStr">
@@ -8576,7 +8576,7 @@
       </c>
       <c r="J141" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.gefahren-baugrundklassen</t>
         </is>
       </c>
     </row>
@@ -8591,7 +8591,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="J142" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
         </is>
       </c>
     </row>
@@ -8639,7 +8639,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -8672,7 +8672,7 @@
       </c>
       <c r="J143" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
         </is>
       </c>
     </row>
@@ -8687,7 +8687,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="J144" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
         </is>
       </c>
     </row>
@@ -8731,21 +8731,21 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Bahnlärm Tag</t>
+          <t>Strassenlärm Tag</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>ch.bafu.laerm-bahnlaerm_tag</t>
+          <t>ch.bafu.laerm-strassenlaerm_tag</t>
         </is>
       </c>
       <c r="F145" s="94" t="inlineStr">
@@ -8768,7 +8768,7 @@
       </c>
       <c r="J145" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-bahnlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-strassenlaerm_tag</t>
         </is>
       </c>
     </row>
@@ -8783,7 +8783,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -8816,7 +8816,7 @@
       </c>
       <c r="J146" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-bahnlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-bahnlaerm_tag</t>
         </is>
       </c>
     </row>
@@ -8831,7 +8831,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="J147" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-bahnlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-bahnlaerm_tag</t>
         </is>
       </c>
     </row>
@@ -8879,7 +8879,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -8912,7 +8912,7 @@
       </c>
       <c r="J148" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-bahnlaerm_tag</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-bahnlaerm_tag</t>
         </is>
       </c>
     </row>
@@ -8923,21 +8923,21 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Hitzebelastung / Klimaanalyse</t>
+          <t>Bahnlärm Tag</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ch.bafu.laerm-bahnlaerm_tag</t>
         </is>
       </c>
       <c r="F149" s="94" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten); keine eindeutige Layer-ID; Link zeigt die Gemeinde ohne Layer</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
         </is>
       </c>
       <c r="H149" t="n">
@@ -8960,7 +8960,7 @@
       </c>
       <c r="J149" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bafu.laerm-bahnlaerm_tag</t>
         </is>
       </c>
     </row>
@@ -8975,7 +8975,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -9008,7 +9008,7 @@
       </c>
       <c r="J150" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -9023,7 +9023,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -9056,7 +9056,7 @@
       </c>
       <c r="J151" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -9071,7 +9071,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="J152" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -9115,16 +9115,16 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Störfall-Risikokataster / belastete Standorte</t>
+          <t>Hitzebelastung / Klimaanalyse</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -9152,7 +9152,7 @@
       </c>
       <c r="J153" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -9167,7 +9167,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -9200,7 +9200,7 @@
       </c>
       <c r="J154" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -9215,7 +9215,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -9248,7 +9248,7 @@
       </c>
       <c r="J155" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -9263,7 +9263,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="J156" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -9307,21 +9307,21 @@
         </is>
       </c>
       <c r="B157" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>ISOS – Ortsbilder von nationaler Bedeutung</t>
+          <t>Störfall-Risikokataster / belastete Standorte</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F157" s="94" t="inlineStr">
@@ -9331,7 +9331,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten); keine eindeutige Layer-ID; Link zeigt die Gemeinde ohne Layer</t>
         </is>
       </c>
       <c r="H157" t="n">
@@ -9344,7 +9344,7 @@
       </c>
       <c r="J157" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau</t>
         </is>
       </c>
     </row>
@@ -9359,7 +9359,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="J158" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
         </is>
       </c>
     </row>
@@ -9407,7 +9407,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -9440,7 +9440,7 @@
       </c>
       <c r="J159" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
         </is>
       </c>
     </row>
@@ -9455,7 +9455,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -9488,7 +9488,7 @@
       </c>
       <c r="J160" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
         </is>
       </c>
     </row>
@@ -9499,21 +9499,21 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>IVS – Historische Verkehrswege (national)</t>
+          <t>ISOS – Ortsbilder von nationaler Bedeutung</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>ch.astra.ivs-nat</t>
+          <t>ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
         </is>
       </c>
       <c r="F161" s="94" t="inlineStr">
@@ -9536,7 +9536,7 @@
       </c>
       <c r="J161" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.bak.bundesinventar-schuetzenswerte-ortsbilder</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -9584,7 +9584,7 @@
       </c>
       <c r="J162" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
         </is>
       </c>
     </row>
@@ -9599,7 +9599,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -9632,7 +9632,7 @@
       </c>
       <c r="J163" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9647,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -9680,7 +9680,7 @@
       </c>
       <c r="J164" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
         </is>
       </c>
     </row>
@@ -9691,21 +9691,21 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>KGS-Inventar (Kulturgüter von nationaler/regionaler Bedeutung)</t>
+          <t>IVS – Historische Verkehrswege (national)</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>ch.babs.kulturgueter</t>
+          <t>ch.astra.ivs-nat</t>
         </is>
       </c>
       <c r="F165" s="94" t="inlineStr">
@@ -9728,7 +9728,7 @@
       </c>
       <c r="J165" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.astra.ivs-nat</t>
         </is>
       </c>
     </row>
@@ -9743,7 +9743,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -9776,7 +9776,7 @@
       </c>
       <c r="J166" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2660000,1190000&amp;z=1&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
         </is>
       </c>
     </row>
@@ -9791,7 +9791,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -9824,7 +9824,7 @@
       </c>
       <c r="J167" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2613308,1263110&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
         </is>
       </c>
     </row>
@@ -9839,7 +9839,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -9872,7 +9872,7 @@
       </c>
       <c r="J168" s="95" t="inlineStr">
         <is>
-          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2721138,1258009&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
         </is>
       </c>
     </row>
@@ -9883,21 +9883,21 @@
         </is>
       </c>
       <c r="B169" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Naturgefahrenkarten BL (Überschwemmung, Murgang, Steinschlag, Rutschung)</t>
+          <t>KGS-Inventar (Kulturgüter von nationaler/regionaler Bedeutung)</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ch.babs.kulturgueter</t>
         </is>
       </c>
       <c r="F169" s="94" t="inlineStr">
@@ -9907,7 +9907,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>Koordinaten lagen bei Liestal; auf Münchenstein gesetzt</t>
+          <t>Hyperlink führte nur auf https://map.geo.admin.ch/ (Layer und Ausschnitt fehlten)</t>
         </is>
       </c>
       <c r="H169" t="n">
@@ -9915,12 +9915,12 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>https://geoview.bl.ch/?map_x=2621744.3974429&amp;map_y=1259205.5204744&amp;map_zoom=4&amp;baselayer_opacity=100&amp;baselayer_ref=grundkarte_farbig&amp;tree_group_layers_Naturgefahren=ghk_wassergefahren_ueberschwemmung_wildbach%2Cghk_wassergefahren_ueberschwemmung_talfluesse</t>
+          <t>https://map.geo.admin.ch/</t>
         </is>
       </c>
       <c r="J169" s="95" t="inlineStr">
         <is>
-          <t>https://geoview.bl.ch/?map_x=2613308&amp;map_y=1263110&amp;map_zoom=4&amp;baselayer_opacity=100&amp;baselayer_ref=grundkarte_farbig&amp;tree_group_layers_Naturgefahren=ghk_wassergefahren_ueberschwemmung_wildbach%2Cghk_wassergefahren_ueberschwemmung_talfluesse</t>
+          <t>https://map.geo.admin.ch/#/map?lang=de&amp;center=2687333,1203124&amp;z=9&amp;bgLayer=ch.swisstopo.pixelkarte-grau&amp;layers=ch.babs.kulturgueter</t>
         </is>
       </c>
     </row>
@@ -9931,16 +9931,16 @@
         </is>
       </c>
       <c r="B170" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Naturgefahrenkarten SG (Geoportal SG)</t>
+          <t>Naturgefahrenkarten BL (Überschwemmung, Murgang, Steinschlag, Rutschung)</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Kartenzentrum lag rund 6 km südlich von Wil; auf Wil zentriert</t>
+          <t>Koordinaten lagen bei Liestal; auf Münchenstein gesetzt</t>
         </is>
       </c>
       <c r="H170" t="n">
@@ -9963,12 +9963,12 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>https://www.geoportal.ch/ktsg/map/3502?y=2717572.22&amp;x=1252351.20&amp;scale=50000&amp;rotation=0</t>
+          <t>https://geoview.bl.ch/?map_x=2621744.3974429&amp;map_y=1259205.5204744&amp;map_zoom=4&amp;baselayer_opacity=100&amp;baselayer_ref=grundkarte_farbig&amp;tree_group_layers_Naturgefahren=ghk_wassergefahren_ueberschwemmung_wildbach%2Cghk_wassergefahren_ueberschwemmung_talfluesse</t>
         </is>
       </c>
       <c r="J170" s="95" t="inlineStr">
         <is>
-          <t>https://www.geoportal.ch/ktsg/map/3502?y=2721138&amp;x=1258009&amp;scale=50000&amp;rotation=0</t>
+          <t>https://geoview.bl.ch/?map_x=2613308&amp;map_y=1263110&amp;map_zoom=4&amp;baselayer_opacity=100&amp;baselayer_ref=grundkarte_farbig&amp;tree_group_layers_Naturgefahren=ghk_wassergefahren_ueberschwemmung_wildbach%2Cghk_wassergefahren_ueberschwemmung_talfluesse</t>
         </is>
       </c>
     </row>
@@ -9979,16 +9979,16 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Geoportal Uri: Nutzungsplanung, Schutzinventare, Naturgefahrenkarten (Seelisberg)</t>
+          <t>Naturgefahrenkarten SG (Geoportal SG)</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -10003,7 +10003,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>URL war beschädigt («¢er», abgeschnittener Parameter) und Lat/Lng lag bei Altdorf; auf Seelisberg gesetzt</t>
+          <t>Kartenzentrum lag rund 6 km südlich von Wil; auf Wil zentriert</t>
         </is>
       </c>
       <c r="H171" t="n">
@@ -10011,47 +10011,47 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>https://geo.ur.ch/?Lat=46.85717868779396&amp;Layers=Nutzungsplanung%2CLiegenschaften%2CBaulanddatenbank&amp;Lng=8.660831451416016&amp;Opacity=0%2C0.4%2C1&amp;Visibility=1%2C1%2C1&amp;Zoom=13¢er%3D955909%2C5937458&amp;center=955830%2C5937741&amp;layers=Nutzungsplanung%20%28Planproduk</t>
+          <t>https://www.geoportal.ch/ktsg/map/3502?y=2717572.22&amp;x=1252351.20&amp;scale=50000&amp;rotation=0</t>
         </is>
       </c>
       <c r="J171" s="95" t="inlineStr">
         <is>
-          <t>https://geo.ur.ch/?Lat=46.9735&amp;Layers=Nutzungsplanung%2CLiegenschaften%2CBaulanddatenbank&amp;Lng=8.5868&amp;Opacity=0%2C0.4%2C1&amp;Visibility=1%2C1%2C1&amp;Zoom=14</t>
+          <t>https://www.geoportal.ch/ktsg/map/3502?y=2721138&amp;x=1258009&amp;scale=50000&amp;rotation=0</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>1_Q1_Rechtsordnung</t>
+          <t>7_GIS_Layers</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Verordnung betreffend den Schutz von Naturkörpern und Altertümern</t>
+          <t>Geoportal Uri: Nutzungsplanung, Schutzinventare, Naturgefahrenkarten (Seelisberg)</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>sGS 271.51</t>
-        </is>
-      </c>
-      <c r="F172" s="96" t="inlineStr">
-        <is>
-          <t>geprüft · manuell prüfen</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F172" s="94" t="inlineStr">
+        <is>
+          <t>geprüft · korrigiert</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Link passt zu Bezeichnung/Referenz, aber Erlass 271.51 «Verordnung betreffend den Schutz von Naturkörpern und Altertümern» ist aufgehoben (vom 21.03.1933, in Vollzug von 21.03.1933 bis: 31.07.2019); Nachfolgeerlass vermutlich sGS 271.53 «Verordnung über die Sicherung und Überlieferung von Naturkörpern» – bitte fachlich bestätigen</t>
+          <t>URL war beschädigt («¢er», abgeschnittener Parameter) und Lat/Lng lag bei Altdorf; auf Seelisberg gesetzt</t>
         </is>
       </c>
       <c r="H172" t="n">
@@ -10059,10 +10059,14 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/271.51</t>
-        </is>
-      </c>
-      <c r="J172" t="inlineStr"/>
+          <t>https://geo.ur.ch/?Lat=46.85717868779396&amp;Layers=Nutzungsplanung%2CLiegenschaften%2CBaulanddatenbank&amp;Lng=8.660831451416016&amp;Opacity=0%2C0.4%2C1&amp;Visibility=1%2C1%2C1&amp;Zoom=13¢er%3D955909%2C5937458&amp;center=955830%2C5937741&amp;layers=Nutzungsplanung%20%28Planproduk</t>
+        </is>
+      </c>
+      <c r="J172" s="95" t="inlineStr">
+        <is>
+          <t>https://geo.ur.ch/?Lat=46.9735&amp;Layers=Nutzungsplanung%2CLiegenschaften%2CBaulanddatenbank&amp;Lng=8.5868&amp;Opacity=0%2C0.4%2C1&amp;Visibility=1%2C1%2C1&amp;Zoom=14</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -16482,6 +16486,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J169" r:id="rId165"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J170" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J171" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J172" r:id="rId168"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21268,9 +21273,9 @@
           <t>Verordnung betreffend den Schutz von Naturkörpern und Altertümern</t>
         </is>
       </c>
-      <c r="E64" s="68" t="inlineStr">
-        <is>
-          <t>sGS 271.51</t>
+      <c r="E64" s="78" t="inlineStr">
+        <is>
+          <t>sGS 271.53</t>
         </is>
       </c>
       <c r="F64" s="68" t="inlineStr">
@@ -21308,14 +21313,14 @@
           <t>Schutz von Altertümern (Archäologie/Denkmal)</t>
         </is>
       </c>
-      <c r="M64" s="72" t="inlineStr">
-        <is>
-          <t>https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/271.51</t>
-        </is>
-      </c>
-      <c r="N64" s="80" t="inlineStr">
-        <is>
-          <t>Muster · geprüft · manuell prüfen</t>
+      <c r="M64" s="74" t="inlineStr">
+        <is>
+          <t>https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/271.53</t>
+        </is>
+      </c>
+      <c r="N64" s="75" t="inlineStr">
+        <is>
+          <t>geprüft · korrigiert</t>
         </is>
       </c>
       <c r="O64" s="68" t="inlineStr">
@@ -21325,7 +21330,7 @@
       </c>
       <c r="P64" s="68" t="inlineStr">
         <is>
-          <t>Nummer aus Gemeinde-Schutzverordnung belegt; Geltung beim Klick prüfen | Linkprüfung 14.10.2026: Link passt zu Bezeichnung/Referenz, aber Erlass 271.51 «Verordnung betreffend den Schutz von Naturkörpern und Altertümern» ist aufgehoben (vom 21.03.1933, in Vollzug von 21.03.1933 bis: 31.07.2019) | Nachfolgeerlass vermutlich sGS 271.53 «Verordnung über die Sicherung und Überlieferung von Naturkörpern» – bitte fachlich bestätigen</t>
+          <t>Nummer aus Gemeinde-Schutzverordnung belegt; Geltung beim Klick prüfen | Linkprüfung 14.10.2026: sGS 271.51 ist seit 31.07.2019 aufgehoben; ersetzt durch den Nachfolgeerlass sGS 271.53 (Titel lt. Sammlung: «Verordnung über die Sicherung und Überlieferung von Naturkörpern»). Alter Link: https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/271.51 | Referenz alt: sGS 271.51</t>
         </is>
       </c>
       <c r="Q64" s="68" t="n"/>
@@ -23874,7 +23879,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" display="https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/841.1" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" display="https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/671.1" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" display="https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/271.51" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" display="https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/841.51" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" display="https://www.gesetzessammlung.sg.ch/app/de/texts_of_law/841.1" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" display="https://rechtsbuch.ur.ch/app/de/texts_of_law/40.1111" r:id="rId58"/>

</xml_diff>